<commit_message>
testing excel uploads, making changes to backend for better error message display
</commit_message>
<xml_diff>
--- a/frontend/public/templates/students_template.xlsx
+++ b/frontend/public/templates/students_template.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t>username</t>
   </si>
@@ -80,13 +80,19 @@
   </si>
   <si>
     <t>family_name</t>
+  </si>
+  <si>
+    <t>is_student</t>
+  </si>
+  <si>
+    <t>is_alumni</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -95,6 +101,11 @@
     </font>
     <font>
       <b/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -114,11 +125,14 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
@@ -354,16 +368,16 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
       <c r="K1" s="1" t="s">
@@ -378,7 +392,7 @@
       <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
       <c r="P1" s="1" t="s">
@@ -393,21 +407,25 @@
       <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" s="2" t="s">
         <v>21</v>
       </c>
       <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="X1" s="2"/>
-      <c r="Y1" s="2"/>
-      <c r="Z1" s="2"/>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="Z1" s="3"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>